<commit_message>
Refactor: per-capita maps, unit scaling, translations (Feb 2026)
</commit_message>
<xml_diff>
--- a/config/impacts.xlsx
+++ b/config/impacts.xlsx
@@ -1,28 +1,31 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jonas\Documents\Hector\Kooperationsphase IO-Modelle\exiobase_explorer\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80421604-DB92-459D-B11F-29868E9B652F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5E94689-B9E4-4779-B2FB-92E4F4C31FBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Exiobase" sheetId="1" r:id="rId1"/>
     <sheet name="color" sheetId="3" r:id="rId2"/>
     <sheet name="Deutsch" sheetId="2" r:id="rId3"/>
+    <sheet name="English" sheetId="4" r:id="rId4"/>
+    <sheet name="Français" sheetId="5" r:id="rId5"/>
+    <sheet name="Español" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="508" uniqueCount="262">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="889" uniqueCount="510">
   <si>
     <t>impact</t>
   </si>
@@ -808,6 +811,750 @@
   </si>
   <si>
     <t>#5ea545</t>
+  </si>
+  <si>
+    <t>Water Consumption Total</t>
+  </si>
+  <si>
+    <t>Valeur ajoutée</t>
+  </si>
+  <si>
+    <t>Emploi</t>
+  </si>
+  <si>
+    <t>Temps de travail</t>
+  </si>
+  <si>
+    <t>Émissions de GES</t>
+  </si>
+  <si>
+    <t>Toxicité humaine</t>
+  </si>
+  <si>
+    <t>Écotoxicité eau douce</t>
+  </si>
+  <si>
+    <t>EPS (dommages)</t>
+  </si>
+  <si>
+    <t>Effets cancérogènes sur la santé (H.A)</t>
+  </si>
+  <si>
+    <t>Maladies respiratoires (organiques) (H.A)</t>
+  </si>
+  <si>
+    <t>Maladies respiratoires (inorganiques) (H.A)</t>
+  </si>
+  <si>
+    <t>Dommages santé liés au climat (H.A)</t>
+  </si>
+  <si>
+    <t>Dommages écosystèmes dus aux substances toxiques (H.A)</t>
+  </si>
+  <si>
+    <t>Dommages par acidification &amp; eutrophisation (H.A)</t>
+  </si>
+  <si>
+    <t>Effets cancérogènes sur la santé (E.E)</t>
+  </si>
+  <si>
+    <t>Maladies respiratoires (organiques) (E.E)</t>
+  </si>
+  <si>
+    <t>Maladies respiratoires (inorganiques) (E.E)</t>
+  </si>
+  <si>
+    <t>Dommages santé liés au climat (E.E)</t>
+  </si>
+  <si>
+    <t>Dommages écosystèmes dus aux substances toxiques (E.E)</t>
+  </si>
+  <si>
+    <t>Dommages par acidification &amp; eutrophisation (E.E)</t>
+  </si>
+  <si>
+    <t>Effets cancérogènes sur la santé (I.I)</t>
+  </si>
+  <si>
+    <t>Maladies respiratoires (organiques) (I.I)</t>
+  </si>
+  <si>
+    <t>Maladies respiratoires (inorganiques) (I.I)</t>
+  </si>
+  <si>
+    <t>Dommages santé liés au climat (I.I)</t>
+  </si>
+  <si>
+    <t>Dommages écosystèmes dus aux substances toxiques (I.I)</t>
+  </si>
+  <si>
+    <t>Dommages par acidification &amp; eutrophisation (I.I)</t>
+  </si>
+  <si>
+    <t>Extraction de matières non utilisée</t>
+  </si>
+  <si>
+    <t>Consommation d’eau verte – agriculture</t>
+  </si>
+  <si>
+    <t>Consommation d’eau bleue – agriculture</t>
+  </si>
+  <si>
+    <t>Consommation d’eau bleue – élevage</t>
+  </si>
+  <si>
+    <t>Consommation d’eau bleue – industrie</t>
+  </si>
+  <si>
+    <t>Consommation d’eau bleue – production d’électricité</t>
+  </si>
+  <si>
+    <t>Consommation d’eau bleue – ménages</t>
+  </si>
+  <si>
+    <t>Consommation d’eau (totale)</t>
+  </si>
+  <si>
+    <t>Prélèvement d’eau bleue – industrie</t>
+  </si>
+  <si>
+    <t>Prélèvement d’eau bleue – production d’électricité</t>
+  </si>
+  <si>
+    <t>Prélèvement d’eau bleue – ménages</t>
+  </si>
+  <si>
+    <t>Prélèvement d’eau bleue – total</t>
+  </si>
+  <si>
+    <t>CO₂ (IPCC cat. 1–4 &amp; 6–7, hors UTCATF)</t>
+  </si>
+  <si>
+    <t>CH₄ (IPCC cat. 1–4 &amp; 6–7, hors UTCATF)</t>
+  </si>
+  <si>
+    <t>N₂O (IPCC cat. 1–4 &amp; 6–7, hors UTCATF)</t>
+  </si>
+  <si>
+    <t>CO₂-éq pour CO₂ (IPCC, hors UTCATF)</t>
+  </si>
+  <si>
+    <t>CO₂-éq pour CH₄ (IPCC, hors UTCATF)</t>
+  </si>
+  <si>
+    <t>CO₂-éq pour N₂O (IPCC, hors UTCATF)</t>
+  </si>
+  <si>
+    <t>CO₂ – combustion &amp; ciment</t>
+  </si>
+  <si>
+    <t>CO₂ – combustion</t>
+  </si>
+  <si>
+    <t>GES (GWP100) – CML 1999 – IPCC 2007</t>
+  </si>
+  <si>
+    <t>GES (GWP100min) – Houghton et al. 2001</t>
+  </si>
+  <si>
+    <t>GES (GWP100max) – Houghton et al. 2001</t>
+  </si>
+  <si>
+    <t>GES (GWP20) – IPCC 2007</t>
+  </si>
+  <si>
+    <t>GES (GWP500) – IPCC 2007</t>
+  </si>
+  <si>
+    <t>Potentiel d’appauvrissement de l’ozone (ODP, état stationnaire)</t>
+  </si>
+  <si>
+    <t>Toxicité humaine (HTP inf) – CML</t>
+  </si>
+  <si>
+    <t>Écotoxicité eau douce (FAETP inf) – CML</t>
+  </si>
+  <si>
+    <t>Écotoxicité marine (MAETP inf) – CML</t>
+  </si>
+  <si>
+    <t>Écotoxicité sédiments eau douce (FSETP inf)</t>
+  </si>
+  <si>
+    <t>Écotoxicité sédiments marins (MSETP inf)</t>
+  </si>
+  <si>
+    <t>Écotoxicité terrestre (TETP inf)</t>
+  </si>
+  <si>
+    <t>Toxicité humaine (HTP20)</t>
+  </si>
+  <si>
+    <t>Écotoxicité eau douce (FAETP20)</t>
+  </si>
+  <si>
+    <t>Écotoxicité marine (MAETP20)</t>
+  </si>
+  <si>
+    <t>Écotoxicité sédiments eau douce (FSETP20)</t>
+  </si>
+  <si>
+    <t>Écotoxicité sédiments marins (MSETP20)</t>
+  </si>
+  <si>
+    <t>Écotoxicité terrestre (TETP20)</t>
+  </si>
+  <si>
+    <t>Toxicité humaine (HTP100)</t>
+  </si>
+  <si>
+    <t>Écotoxicité eau douce (FAETP100)</t>
+  </si>
+  <si>
+    <t>Écotoxicité marine (MAETP100)</t>
+  </si>
+  <si>
+    <t>Écotoxicité sédiments eau douce (FSETP100)</t>
+  </si>
+  <si>
+    <t>Écotoxicité sédiments marins (MSETP100)</t>
+  </si>
+  <si>
+    <t>Écotoxicité terrestre (TETP100)</t>
+  </si>
+  <si>
+    <t>Toxicité humaine (HTP500)</t>
+  </si>
+  <si>
+    <t>Écotoxicité eau douce (FAETP500)</t>
+  </si>
+  <si>
+    <t>Écotoxicité marine (MAETP500)</t>
+  </si>
+  <si>
+    <t>Écotoxicité sédiments eau douce (FSETP500)</t>
+  </si>
+  <si>
+    <t>Toxicité sédiments marins (MSETP500) – alternatif</t>
+  </si>
+  <si>
+    <t>Écotoxicité terrestre (TETP500) – alternatif</t>
+  </si>
+  <si>
+    <t>Oxydation photochimique (NOx élevés) – POCP</t>
+  </si>
+  <si>
+    <t>Oxydation photochimique (NOx faibles) – POCP</t>
+  </si>
+  <si>
+    <t>Oxydation photochimique (MIR)</t>
+  </si>
+  <si>
+    <t>Oxydation photochimique (MOIR)</t>
+  </si>
+  <si>
+    <t>Oxydation photochimique (EBIR)</t>
+  </si>
+  <si>
+    <t>Acidification (avec “sort”/fate)</t>
+  </si>
+  <si>
+    <t>Acidification (sans “sort”/fate)</t>
+  </si>
+  <si>
+    <t>Eutrophisation (sans “sort”/fate)</t>
+  </si>
+  <si>
+    <t>Eutrophisation (avec “sort”/fate)</t>
+  </si>
+  <si>
+    <t>Odeur</t>
+  </si>
+  <si>
+    <t>Changement climatique (moyenne, ILCD) – GWP100</t>
+  </si>
+  <si>
+    <t>CC – endpoint santé humaine (ILCD)</t>
+  </si>
+  <si>
+    <t>CC – endpoint écosystèmes (ILCD)</t>
+  </si>
+  <si>
+    <t>Toxicité humaine (cancer, ILCD)</t>
+  </si>
+  <si>
+    <t>Toxicité humaine (non-cancer, ILCD)</t>
+  </si>
+  <si>
+    <t>Toxicité humaine endpoint (cancer, ILCD)</t>
+  </si>
+  <si>
+    <t>Toxicité humaine endpoint (non-cancer, ILCD)</t>
+  </si>
+  <si>
+    <t>Particules fines / inorganiques resp. (midpoint, ILCD)</t>
+  </si>
+  <si>
+    <t>Particules fines endpoint (ILCD)</t>
+  </si>
+  <si>
+    <t>Ozone photochimique (midpoint, ILCD)</t>
+  </si>
+  <si>
+    <t>Ozone photochimique endpoint (ILCD)</t>
+  </si>
+  <si>
+    <t>Acidification (midpoint, ILCD)</t>
+  </si>
+  <si>
+    <t>Acidification endpoint (ILCD)</t>
+  </si>
+  <si>
+    <t>Eutrophisation terrestre (midpoint, ILCD)</t>
+  </si>
+  <si>
+    <t>Eutrophisation marine (midpoint, ILCD)</t>
+  </si>
+  <si>
+    <t>Écotoxicité eau douce (midpoint, ILCD)</t>
+  </si>
+  <si>
+    <t>Écotoxicité eau douce endpoint (ILCD)</t>
+  </si>
+  <si>
+    <t>GES AR5 (GWP100) – IPCC 2010</t>
+  </si>
+  <si>
+    <t>Azote</t>
+  </si>
+  <si>
+    <t>Phosphore</t>
+  </si>
+  <si>
+    <t>PM2.5</t>
+  </si>
+  <si>
+    <t>Utilisation de l’extraction domestique – récoltes &amp; résidus</t>
+  </si>
+  <si>
+    <t>Utilisation de l’extraction domestique – pâturages &amp; fourrages</t>
+  </si>
+  <si>
+    <t>Utilisation de l’extraction domestique – foresterie &amp; bois</t>
+  </si>
+  <si>
+    <t>Extraction domestique utilisée – pêches</t>
+  </si>
+  <si>
+    <t>Utilisation de l’extraction domestique – minéraux non métalliques</t>
+  </si>
+  <si>
+    <t>Utilisation de l’extraction domestique – minerai de fer</t>
+  </si>
+  <si>
+    <t>Utilisation de l’extraction domestique – minerais non ferreux</t>
+  </si>
+  <si>
+    <t>Extraction domestique non utilisée – récoltes &amp; résidus</t>
+  </si>
+  <si>
+    <t>Extraction domestique non utilisée – pâturages &amp; fourrages</t>
+  </si>
+  <si>
+    <t>Extraction domestique non utilisée – foresterie &amp; bois</t>
+  </si>
+  <si>
+    <t>Extraction domestique non utilisée – pêches</t>
+  </si>
+  <si>
+    <t>Extraction domestique non utilisée – charbon &amp; tourbe</t>
+  </si>
+  <si>
+    <t>Extraction domestique non utilisée – pétrole &amp; gaz</t>
+  </si>
+  <si>
+    <t>Extraction domestique non utilisée – minéraux non métalliques</t>
+  </si>
+  <si>
+    <t>Extraction domestique non utilisée – minerai de fer</t>
+  </si>
+  <si>
+    <t>Extraction domestique non utilisée – minerais non ferreux</t>
+  </si>
+  <si>
+    <t>Occupation des sols</t>
+  </si>
+  <si>
+    <t>Valor añadido</t>
+  </si>
+  <si>
+    <t>Empleo</t>
+  </si>
+  <si>
+    <t>Tiempo de trabajo</t>
+  </si>
+  <si>
+    <t>Emisiones de gases de efecto invernadero</t>
+  </si>
+  <si>
+    <t>Toxicidad humana</t>
+  </si>
+  <si>
+    <t>Ecotoxicidad en agua dulce</t>
+  </si>
+  <si>
+    <t>Enfoque de daños EPS</t>
+  </si>
+  <si>
+    <t>Efectos cancerígenos en humanos (H.A)</t>
+  </si>
+  <si>
+    <t>Enfermedades respiratorias por sustancias orgánicas (H.A)</t>
+  </si>
+  <si>
+    <t>Enfermedades respiratorias por sustancias inorgánicas (H.A)</t>
+  </si>
+  <si>
+    <t>Daños a la salud por cambio climático (H.A)</t>
+  </si>
+  <si>
+    <t>Daños a la calidad de los ecosistemas por sustancias nocivas (H.A)</t>
+  </si>
+  <si>
+    <t>Daños por acidificación y eutrofización (H.A)</t>
+  </si>
+  <si>
+    <t>Efectos cancerígenos en humanos (E.E)</t>
+  </si>
+  <si>
+    <t>Enfermedades respiratorias por sustancias orgánicas (E.E)</t>
+  </si>
+  <si>
+    <t>Enfermedades respiratorias por sustancias inorgánicas (E.E)</t>
+  </si>
+  <si>
+    <t>Daños a la salud por cambio climático (E.E)</t>
+  </si>
+  <si>
+    <t>Daños a la calidad de los ecosistemas por sustancias nocivas (E.E)</t>
+  </si>
+  <si>
+    <t>Daños por acidificación y eutrofización (E.E)</t>
+  </si>
+  <si>
+    <t>Efectos cancerígenos en humanos (I.I)</t>
+  </si>
+  <si>
+    <t>Enfermedades respiratorias por sustancias orgánicas (I.I)</t>
+  </si>
+  <si>
+    <t>Enfermedades respiratorias por sustancias inorgánicas (I.I)</t>
+  </si>
+  <si>
+    <t>Daños a la salud por cambio climático (I.I)</t>
+  </si>
+  <si>
+    <t>Daños a la calidad de los ecosistemas por sustancias nocivas (I.I)</t>
+  </si>
+  <si>
+    <t>Daños por acidificación y eutrofización (I.I)</t>
+  </si>
+  <si>
+    <t>Extracción de recursos no utilizada</t>
+  </si>
+  <si>
+    <t>Consumo de agua verde - agricultura</t>
+  </si>
+  <si>
+    <t>Consumo de agua azul - agricultura</t>
+  </si>
+  <si>
+    <t>Consumo de agua azul - ganadería</t>
+  </si>
+  <si>
+    <t>Consumo de agua azul - industria</t>
+  </si>
+  <si>
+    <t>Consumo de agua azul - generación eléctrica</t>
+  </si>
+  <si>
+    <t>Consumo de agua azul - hogares</t>
+  </si>
+  <si>
+    <t>Consumo de agua</t>
+  </si>
+  <si>
+    <t>Extracción de agua azul - industria</t>
+  </si>
+  <si>
+    <t>Extracción de agua azul - generación eléctrica</t>
+  </si>
+  <si>
+    <t>Extracción de agua azul - hogares</t>
+  </si>
+  <si>
+    <t>Extracción de agua azul - total</t>
+  </si>
+  <si>
+    <t>Dióxido de carbono (CO₂) IPCC categorías 1-4 y 6-7 (sin uso/cambio de uso del suelo y silvicultura)</t>
+  </si>
+  <si>
+    <t>Metano (CH₄) IPCC categorías 1-4 y 6-7 (sin uso/cambio de uso del suelo y silvicultura)</t>
+  </si>
+  <si>
+    <t>Óxido nitroso (N₂O) IPCC categorías 1-4 y 6-7 (sin uso/cambio de uso del suelo y silvicultura)</t>
+  </si>
+  <si>
+    <t>CO₂-equivalente (CO₂eq) para CO₂ IPCC categorías 1-4 y 6-7 (sin uso/cambio de uso del suelo)</t>
+  </si>
+  <si>
+    <t>CO₂-equivalente (CO₂eq) para metano (CH₄) IPCC categorías 1-4 y 6-7 (sin uso/cambio de uso del suelo)</t>
+  </si>
+  <si>
+    <t>CO₂-equivalente (CO₂eq) para óxido nitroso (N₂O) IPCC categorías 1-4 y 6-7 (sin uso/cambio de uso del suelo)</t>
+  </si>
+  <si>
+    <t>Dióxido de carbono (CO₂) procedente de la combustión de combustibles y la producción de cemento</t>
+  </si>
+  <si>
+    <t>Dióxido de carbono (CO₂) procedente de la combustión de combustibles</t>
+  </si>
+  <si>
+    <t>Emisiones de gases de efecto invernadero (GWP100) | Enfoque base (CML, 1999) | GWP100 (IPCC, 2007)</t>
+  </si>
+  <si>
+    <t>Emisiones de gases de efecto invernadero (GWP100min) | Enfoque alternativo | GWP100 neto mín. (Houghton et al., 2001)</t>
+  </si>
+  <si>
+    <t>Emisiones de gases de efecto invernadero (GWP100max) | Enfoque alternativo | GWP100 neto máx. (Houghton et al., 2001)</t>
+  </si>
+  <si>
+    <t>Emisiones de gases de efecto invernadero (GWP20) | Enfoque alternativo | GWP20 (IPCC, 2007)</t>
+  </si>
+  <si>
+    <t>Emisiones de gases de efecto invernadero (GWP500) | Enfoque alternativo | GWP500 (IPCC, 2007)</t>
+  </si>
+  <si>
+    <t>Potencial de agotamiento del ozono (ODP, estado estacionario) | Enfoque orientado al problema: base | ODP, estado estacionario</t>
+  </si>
+  <si>
+    <t>Toxicidad humana (HTP inf) | Enfoque orientado al problema: base</t>
+  </si>
+  <si>
+    <t>Ecotoxicidad en agua dulce (FAETP inf) | Enfoque orientado al problema: base</t>
+  </si>
+  <si>
+    <t>Ecotoxicidad en el medio marino (MAETP inf) | Enfoque orientado al problema: base</t>
+  </si>
+  <si>
+    <t>Ecotoxicidad sedimentaria en agua dulce (FSETP inf) | Enfoque orientado al problema: no base</t>
+  </si>
+  <si>
+    <t>Ecotoxicidad sedimentaria en el medio marino (MSETP inf) | Enfoque orientado al problema: no base</t>
+  </si>
+  <si>
+    <t>Ecotoxicidad terrestre (TETP inf) | Enfoque orientado al problema: base</t>
+  </si>
+  <si>
+    <t>Toxicidad humana (HTP20) | Enfoque orientado al problema: no base</t>
+  </si>
+  <si>
+    <t>Ecotoxicidad en agua dulce (FAETP20) | Enfoque orientado al problema: no base</t>
+  </si>
+  <si>
+    <t>Ecotoxicidad en el medio marino (MAETP20) | Enfoque orientado al problema: no base</t>
+  </si>
+  <si>
+    <t>Ecotoxicidad sedimentaria en agua dulce (FSETP20) | Enfoque orientado al problema: no base</t>
+  </si>
+  <si>
+    <t>Ecotoxicidad sedimentaria en el medio marino (MSETP20) | Enfoque orientado al problema: no base</t>
+  </si>
+  <si>
+    <t>Ecotoxicidad terrestre (TETP20) | Enfoque orientado al problema: no base</t>
+  </si>
+  <si>
+    <t>Toxicidad humana (HTP100) | Enfoque orientado al problema: no base</t>
+  </si>
+  <si>
+    <t>Ecotoxicidad en agua dulce (FAETP100) | Enfoque orientado al problema: no base</t>
+  </si>
+  <si>
+    <t>Ecotoxicidad en el medio marino (MAETP100) | Enfoque orientado al problema: no base</t>
+  </si>
+  <si>
+    <t>Ecotoxicidad sedimentaria en agua dulce (FSETP100) | Enfoque orientado al problema: no base</t>
+  </si>
+  <si>
+    <t>Ecotoxicidad sedimentaria en el medio marino (MSETP100) | Enfoque orientado al problema: no base</t>
+  </si>
+  <si>
+    <t>Ecotoxicidad terrestre (TETP100) | Enfoque orientado al problema: no base</t>
+  </si>
+  <si>
+    <t>Toxicidad humana (HTP500) | Enfoque orientado al problema: no base</t>
+  </si>
+  <si>
+    <t>Ecotoxicidad en agua dulce (FAETP500) | Enfoque orientado al problema: no base</t>
+  </si>
+  <si>
+    <t>Ecotoxicidad en el medio marino (MAETP500) | Enfoque orientado al problema: no base</t>
+  </si>
+  <si>
+    <t>Ecotoxicidad sedimentaria en agua dulce (FSETP500) | Enfoque orientado al problema: no base</t>
+  </si>
+  <si>
+    <t>Toxicidad de sedimentos marinos (MSETP500) | Enfoque alternativo (CML, 1999) | MSETP 500 (Huijbregts, 1999 y 2000)</t>
+  </si>
+  <si>
+    <t>Ecotoxicidad terrestre (TETP500) | Enfoque alternativo (CML, 1999) | TETP 500 (Huijbregts, 1999 y 2000)</t>
+  </si>
+  <si>
+    <t>Oxidación fotoquímica (valores altos de NOx) | Enfoque base (CML, 1999) | POCP (Jenkin y Hayman, 1999; Derwent et al., 1998)</t>
+  </si>
+  <si>
+    <t>Oxidación fotoquímica (valores bajos de NOx) | Enfoque alternativo (CML, 1999) | POCP (Andersson-Sköld et al., 1992)</t>
+  </si>
+  <si>
+    <t>Oxidación fotoquímica (MIR; valores muy altos de NOx) | Enfoque alternativo (CML, 1999) | MIR 1997 (Carter, 1994, 1997, 1998; Carter et al., 1995)</t>
+  </si>
+  <si>
+    <t>Oxidación fotoquímica (MOIR; NOx alto) | Enfoque orientado al problema: no base</t>
+  </si>
+  <si>
+    <t>Oxidación fotoquímica (EBIR; NOx bajo) | Enfoque orientado al problema: no base</t>
+  </si>
+  <si>
+    <t>Acidificación (incl. destino, media Europa total, A&amp;B) | Enfoque orientado al problema: base</t>
+  </si>
+  <si>
+    <t>Acidificación (sin destino) | Enfoque orientado al problema: no base</t>
+  </si>
+  <si>
+    <t>Eutrofización (sin destino) | Enfoque orientado al problema: base</t>
+  </si>
+  <si>
+    <t>Eutrofización (incl. destino, media Europa total, A&amp;B) | Enfoque orientado al problema: no base</t>
+  </si>
+  <si>
+    <t>Olor | Enfoque orientado al problema: no base</t>
+  </si>
+  <si>
+    <t>Cambio climático (promedio) | CF recomendado por ILCD | Potencial de calentamiento global a 100 años</t>
+  </si>
+  <si>
+    <t>Cambio climático (endpoint), salud humana | CF recomendado por ILCD | Años de vida ajustados por discapacidad (DALY)</t>
+  </si>
+  <si>
+    <t>Cambio climático (endpoint), ecosistemas | CF recomendado por ILCD | Fracción de especies potencialmente desaparecidas (PDF)</t>
+  </si>
+  <si>
+    <t>Toxicidad humana (promedio), efectos cancerígenos | CF recomendado por ILCD | Unidad comparativa para toxicidad humana (CTUh)</t>
+  </si>
+  <si>
+    <t>Toxicidad humana (promedio), sin efectos cancerígenos | CF recomendado por ILCD | Unidad comparativa para toxicidad humana (CTUh)</t>
+  </si>
+  <si>
+    <t>Toxicidad humana (endpoint), efectos cancerígenos | CF recomendado por ILCD | Años de vida ajustados por discapacidad (DALY)</t>
+  </si>
+  <si>
+    <t>Toxicidad humana (endpoint), sin efectos cancerígenos | CF recomendado por ILCD | Años de vida ajustados por discapacidad (DALY)</t>
+  </si>
+  <si>
+    <t>Partículas finas / sustancias inorgánicas respiratorias (promedio) | CF recomendado por ILCD | Equivalente medio ponderado por emisiones de PM2,5</t>
+  </si>
+  <si>
+    <t>Partículas finas / sustancias inorgánicas respiratorias (endpoint) | CF recomendado por ILCD | Años de vida ajustados por discapacidad (DALY)</t>
+  </si>
+  <si>
+    <t>Formación de ozono fotoquímico (promedio), salud humana | CF recomendado por ILCD | Potencial de formación de ozono fotoquímico (POCP)</t>
+  </si>
+  <si>
+    <t>Formación de ozono fotoquímico (endpoint), salud humana | CF recomendado por ILCD | Años de vida ajustados por discapacidad (DALY)</t>
+  </si>
+  <si>
+    <t>Acidificación (promedio) | CF recomendado por ILCD | Excedencia acumulada (AE)</t>
+  </si>
+  <si>
+    <t>Acidificación (endpoint) | CF recomendado por ILCD | Cambio en la fracción de especies vegetales potencialmente ausentes por cambio en la saturación de bases</t>
+  </si>
+  <si>
+    <t>Eutrofización terrestre (promedio) | CF recomendado por ILCD | Excedencia acumulada (AE)</t>
+  </si>
+  <si>
+    <t>Eutrofización marina (promedio) | CF recomendado por ILCD | Fracciones de especies potencialmente desaparecidas (PDF)</t>
+  </si>
+  <si>
+    <t>Ecotoxicidad en agua dulce (promedio) | CF recomendado por ILCD | Unidad comparativa para ecosistemas (CTUe)</t>
+  </si>
+  <si>
+    <t>Ecotoxicidad en agua dulce (endpoint) | CF recomendado por ILCD | Fracciones de especies potencialmente desaparecidas (PDF)</t>
+  </si>
+  <si>
+    <t>Emisiones de GEI AR5 (GWP100) | GWP100 (IPCC, 2010)</t>
+  </si>
+  <si>
+    <t>Nitrógeno</t>
+  </si>
+  <si>
+    <t>Fósforo</t>
+  </si>
+  <si>
+    <t>Uso de la extracción doméstica - cosecha y residuos de cosecha</t>
+  </si>
+  <si>
+    <t>Uso de la extracción doméstica - pastos y forraje</t>
+  </si>
+  <si>
+    <t>Uso de la extracción doméstica - silvicultura y madera</t>
+  </si>
+  <si>
+    <t>Extracción doméstica utilizada – pesca</t>
+  </si>
+  <si>
+    <t>Uso de la extracción doméstica - minerales no metálicos</t>
+  </si>
+  <si>
+    <t>Uso de la extracción doméstica - mineral de hierro</t>
+  </si>
+  <si>
+    <t>Uso de la extracción doméstica - minerales de metales no ferrosos</t>
+  </si>
+  <si>
+    <t>Extracción doméstica no utilizada - cosecha y residuos de cosecha</t>
+  </si>
+  <si>
+    <t>Extracción doméstica no utilizada - pastos y forraje</t>
+  </si>
+  <si>
+    <t>Extracción doméstica no utilizada - silvicultura y madera</t>
+  </si>
+  <si>
+    <t>Extracción doméstica no utilizada – pesca</t>
+  </si>
+  <si>
+    <t>Extracción doméstica no utilizada - carbón y turba</t>
+  </si>
+  <si>
+    <t>Extracción doméstica no utilizada - petróleo y gas</t>
+  </si>
+  <si>
+    <t>Extracción doméstica no utilizada - minerales no metálicos</t>
+  </si>
+  <si>
+    <t>Extracción doméstica no utilizada - mineral de hierro</t>
+  </si>
+  <si>
+    <t>Extracción doméstica no utilizada - minerales de metales no ferrosos</t>
+  </si>
+  <si>
+    <t>Uso del suelo</t>
+  </si>
+  <si>
+    <t>Indicador ambiental</t>
+  </si>
+  <si>
+    <t>Indicateur environnemental</t>
   </si>
 </sst>
 </file>
@@ -3511,4 +4258,1948 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{73350C52-5375-4581-B197-23D075092142}">
+  <dimension ref="A1:A127"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="209.85546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A8" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A9" s="3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A10" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A11" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A12" s="3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A13" s="3" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A14" s="3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A15" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A16" s="3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A17" s="3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A18" s="3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A19" s="3" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A20" s="3" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A21" s="3" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A22" s="3" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A23" s="3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A24" s="3" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A25" s="3" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A26" s="3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A27" s="3" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A28" s="3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A29" s="3" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A30" s="3" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A31" s="3" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A32" s="3" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A33" s="3" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A34" s="3" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A35" s="3" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A36" s="3" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A37" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A38" s="3" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A39" s="3" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A40" s="3" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="41" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A41" s="3" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A42" s="3" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="43" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A43" s="3" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="44" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A44" s="3" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="45" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A45" s="3" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="46" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A46" s="3" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="47" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A47" s="3" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="48" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A48" s="3" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="49" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A49" s="3" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="50" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A50" s="3" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="51" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A51" s="3" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="52" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A52" s="3" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="53" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A53" s="3" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="54" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A54" s="3" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="55" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A55" s="3" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="56" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A56" s="3" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="57" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A57" s="3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="58" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A58" s="3" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="59" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A59" s="3" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="60" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A60" s="3" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="61" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A61" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="62" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A62" s="3" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="63" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A63" s="3" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="64" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A64" s="3" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="65" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A65" s="3" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="66" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A66" s="3" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="67" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A67" s="3" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="68" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A68" s="3" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="69" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A69" s="3" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="70" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A70" s="3" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="71" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A71" s="3" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="72" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A72" s="3" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="73" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A73" s="3" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="74" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A74" s="3" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="75" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A75" s="3" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="76" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A76" s="3" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="77" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A77" s="3" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="78" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A78" s="3" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="79" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A79" s="3" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="80" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A80" s="3" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="81" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A81" s="3" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="82" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A82" s="3" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="83" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A83" s="3" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="84" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A84" s="3" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="85" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A85" s="3" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="86" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A86" s="3" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="87" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A87" s="3" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="88" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A88" s="3" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="89" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A89" s="3" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="90" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A90" s="3" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="91" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A91" s="3" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="92" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A92" s="3" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="93" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A93" s="3" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="94" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A94" s="3" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="95" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A95" s="3" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="96" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A96" s="3" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="97" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A97" s="3" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="98" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A98" s="3" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="99" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A99" s="3" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="100" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A100" s="3" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="101" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A101" s="3" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="102" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A102" s="3" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="103" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A103" s="3" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="104" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A104" s="3" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="105" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A105" s="3" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="106" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A106" s="3" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="107" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A107" s="3" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="108" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A108" s="3" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="109" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A109" s="3" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="110" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A110" s="3" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="111" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A111" s="3" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="112" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A112" s="3" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="113" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A113" s="3" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="114" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A114" s="3" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="115" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A115" s="3" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="116" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A116" s="3" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="117" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A117" s="3" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="118" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A118" s="3" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="119" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A119" s="3" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="120" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A120" s="3" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="121" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A121" s="3" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="122" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A122" s="3" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="123" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A123" s="3" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="124" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A124" s="3" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="125" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A125" s="3" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="126" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A126" s="3" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="127" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A127" s="3" t="s">
+        <v>126</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{540A48AF-DC29-4294-9986-F1C6AE7ABB75}">
+  <dimension ref="A1:A127"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="61" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>509</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A8" s="3" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A9" s="3" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A10" s="3" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A11" s="3" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A12" s="3" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A13" s="3" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A14" s="3" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A15" s="3" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A16" s="3" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A17" s="3" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A18" s="3" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A19" s="3" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A20" s="3" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A21" s="3" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A22" s="3" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A23" s="3" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A24" s="3" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A25" s="3" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A26" s="3" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A27" s="3" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A28" s="3" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A29" s="3" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A30" s="3" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A31" s="3" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A32" s="3" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A33" s="3" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A34" s="3" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A35" s="3" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A36" s="3" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A37" s="3" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A38" s="3" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A39" s="3" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A40" s="3" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="41" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A41" s="3" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A42" s="3" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="43" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A43" s="3" t="s">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="44" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A44" s="3" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="45" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A45" s="3" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="46" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A46" s="3" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="47" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A47" s="3" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="48" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A48" s="3" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="49" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A49" s="3" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="50" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A50" s="3" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="51" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A51" s="3" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="52" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A52" s="3" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="53" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A53" s="3" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="54" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A54" s="3" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="55" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A55" s="3" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="56" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A56" s="3" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="57" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A57" s="3" t="s">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="58" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A58" s="3" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="59" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A59" s="3" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="60" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A60" s="3" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="61" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A61" s="3" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="62" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A62" s="3" t="s">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="63" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A63" s="3" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="64" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A64" s="3" t="s">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="65" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A65" s="3" t="s">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="66" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A66" s="3" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="67" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A67" s="3" t="s">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="68" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A68" s="3" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="69" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A69" s="3" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="70" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A70" s="3" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="71" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A71" s="3" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="72" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A72" s="3" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="73" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A73" s="3" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="74" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A74" s="3" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="75" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A75" s="3" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="76" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A76" s="3" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="77" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A77" s="3" t="s">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="78" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A78" s="3" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="79" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A79" s="3" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="80" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A80" s="3" t="s">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="81" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A81" s="3" t="s">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="82" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A82" s="3" t="s">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="83" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A83" s="3" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="84" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A84" s="3" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="85" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A85" s="3" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="86" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A86" s="3" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="87" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A87" s="3" t="s">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="88" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A88" s="3" t="s">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="89" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A89" s="3" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="90" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A90" s="3" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="91" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A91" s="3" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="92" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A92" s="3" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="93" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A93" s="3" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="94" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A94" s="3" t="s">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="95" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A95" s="3" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="96" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A96" s="3" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="97" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A97" s="3" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="98" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A98" s="3" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="99" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A99" s="3" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="100" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A100" s="3" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="101" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A101" s="3" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="102" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A102" s="3" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="103" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A103" s="3" t="s">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="104" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A104" s="3" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="105" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A105" s="3" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="106" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A106" s="3" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="107" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A107" s="3" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="108" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A108" s="3" t="s">
+        <v>368</v>
+      </c>
+    </row>
+    <row r="109" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A109" s="3" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="110" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A110" s="3" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="111" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A111" s="3" t="s">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="112" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A112" s="3" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="113" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A113" s="3" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="114" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A114" s="3" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="115" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A115" s="3" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="116" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A116" s="3" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="117" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A117" s="3" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="118" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A118" s="3" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="119" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A119" s="3" t="s">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="120" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A120" s="3" t="s">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="121" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A121" s="3" t="s">
+        <v>379</v>
+      </c>
+    </row>
+    <row r="122" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A122" s="3" t="s">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="123" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A123" s="3" t="s">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="124" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A124" s="3" t="s">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="125" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A125" s="3" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="126" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A126" s="3" t="s">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="127" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A127" s="3" t="s">
+        <v>385</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{33B5C7DE-6334-42C5-8830-061C71A1999D}">
+  <dimension ref="A1:A127"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="146.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>508</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A8" s="3" t="s">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A9" s="3" t="s">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A10" s="3" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A11" s="3" t="s">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A12" s="3" t="s">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A13" s="3" t="s">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A14" s="3" t="s">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A15" s="3" t="s">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A16" s="3" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A17" s="3" t="s">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A18" s="3" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A19" s="3" t="s">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A20" s="3" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A21" s="3" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A22" s="3" t="s">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A23" s="3" t="s">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A24" s="3" t="s">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A25" s="3" t="s">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A26" s="3" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A27" s="3" t="s">
+        <v>411</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A28" s="3" t="s">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A29" s="3" t="s">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A30" s="3" t="s">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A31" s="3" t="s">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A32" s="3" t="s">
+        <v>416</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A33" s="3" t="s">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A34" s="3" t="s">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A35" s="3" t="s">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A36" s="3" t="s">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A37" s="3" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A38" s="3" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A39" s="3" t="s">
+        <v>423</v>
+      </c>
+    </row>
+    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A40" s="3" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="41" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A41" s="3" t="s">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A42" s="3" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="43" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A43" s="3" t="s">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="44" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A44" s="3" t="s">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="45" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A45" s="3" t="s">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="46" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A46" s="3" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="47" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A47" s="3" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="48" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A48" s="3" t="s">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="49" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A49" s="3" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="50" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A50" s="3" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="51" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A51" s="3" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="52" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A52" s="3" t="s">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="53" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A53" s="3" t="s">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="54" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A54" s="3" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="55" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A55" s="3" t="s">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="56" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A56" s="3" t="s">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="57" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A57" s="3" t="s">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="58" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A58" s="3" t="s">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="59" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A59" s="3" t="s">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="60" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A60" s="3" t="s">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="61" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A61" s="3" t="s">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="62" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A62" s="3" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="63" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A63" s="3" t="s">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="64" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A64" s="3" t="s">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="65" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A65" s="3" t="s">
+        <v>449</v>
+      </c>
+    </row>
+    <row r="66" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A66" s="3" t="s">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="67" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A67" s="3" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="68" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A68" s="3" t="s">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="69" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A69" s="3" t="s">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="70" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A70" s="3" t="s">
+        <v>454</v>
+      </c>
+    </row>
+    <row r="71" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A71" s="3" t="s">
+        <v>455</v>
+      </c>
+    </row>
+    <row r="72" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A72" s="3" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="73" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A73" s="3" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="74" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A74" s="3" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="75" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A75" s="3" t="s">
+        <v>459</v>
+      </c>
+    </row>
+    <row r="76" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A76" s="3" t="s">
+        <v>460</v>
+      </c>
+    </row>
+    <row r="77" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A77" s="3" t="s">
+        <v>461</v>
+      </c>
+    </row>
+    <row r="78" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A78" s="3" t="s">
+        <v>462</v>
+      </c>
+    </row>
+    <row r="79" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A79" s="3" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="80" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A80" s="3" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="81" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A81" s="3" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="82" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A82" s="3" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="83" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A83" s="3" t="s">
+        <v>467</v>
+      </c>
+    </row>
+    <row r="84" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A84" s="3" t="s">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="85" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A85" s="3" t="s">
+        <v>469</v>
+      </c>
+    </row>
+    <row r="86" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A86" s="3" t="s">
+        <v>470</v>
+      </c>
+    </row>
+    <row r="87" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A87" s="3" t="s">
+        <v>471</v>
+      </c>
+    </row>
+    <row r="88" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A88" s="3" t="s">
+        <v>472</v>
+      </c>
+    </row>
+    <row r="89" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A89" s="3" t="s">
+        <v>473</v>
+      </c>
+    </row>
+    <row r="90" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A90" s="3" t="s">
+        <v>474</v>
+      </c>
+    </row>
+    <row r="91" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A91" s="3" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="92" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A92" s="3" t="s">
+        <v>476</v>
+      </c>
+    </row>
+    <row r="93" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A93" s="3" t="s">
+        <v>477</v>
+      </c>
+    </row>
+    <row r="94" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A94" s="3" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="95" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A95" s="3" t="s">
+        <v>479</v>
+      </c>
+    </row>
+    <row r="96" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A96" s="3" t="s">
+        <v>480</v>
+      </c>
+    </row>
+    <row r="97" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A97" s="3" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="98" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A98" s="3" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="99" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A99" s="3" t="s">
+        <v>483</v>
+      </c>
+    </row>
+    <row r="100" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A100" s="3" t="s">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="101" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A101" s="3" t="s">
+        <v>485</v>
+      </c>
+    </row>
+    <row r="102" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A102" s="3" t="s">
+        <v>486</v>
+      </c>
+    </row>
+    <row r="103" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A103" s="3" t="s">
+        <v>487</v>
+      </c>
+    </row>
+    <row r="104" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A104" s="3" t="s">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="105" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A105" s="3" t="s">
+        <v>489</v>
+      </c>
+    </row>
+    <row r="106" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A106" s="3" t="s">
+        <v>490</v>
+      </c>
+    </row>
+    <row r="107" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A107" s="3" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="108" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A108" s="3" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="109" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A109" s="3" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="110" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A110" s="3" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="111" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A111" s="3" t="s">
+        <v>491</v>
+      </c>
+    </row>
+    <row r="112" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A112" s="3" t="s">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="113" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A113" s="3" t="s">
+        <v>493</v>
+      </c>
+    </row>
+    <row r="114" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A114" s="3" t="s">
+        <v>494</v>
+      </c>
+    </row>
+    <row r="115" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A115" s="3" t="s">
+        <v>495</v>
+      </c>
+    </row>
+    <row r="116" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A116" s="3" t="s">
+        <v>496</v>
+      </c>
+    </row>
+    <row r="117" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A117" s="3" t="s">
+        <v>497</v>
+      </c>
+    </row>
+    <row r="118" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A118" s="3" t="s">
+        <v>498</v>
+      </c>
+    </row>
+    <row r="119" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A119" s="3" t="s">
+        <v>499</v>
+      </c>
+    </row>
+    <row r="120" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A120" s="3" t="s">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="121" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A121" s="3" t="s">
+        <v>501</v>
+      </c>
+    </row>
+    <row r="122" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A122" s="3" t="s">
+        <v>502</v>
+      </c>
+    </row>
+    <row r="123" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A123" s="3" t="s">
+        <v>503</v>
+      </c>
+    </row>
+    <row r="124" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A124" s="3" t="s">
+        <v>504</v>
+      </c>
+    </row>
+    <row r="125" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A125" s="3" t="s">
+        <v>505</v>
+      </c>
+    </row>
+    <row r="126" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A126" s="3" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="127" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A127" s="3" t="s">
+        <v>507</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>